<commit_message>
update to raw data packages
</commit_message>
<xml_diff>
--- a/Ontario/Raw Data/Ontario 2023 NS for Chris Oct 8.xlsx
+++ b/Ontario/Raw Data/Ontario 2023 NS for Chris Oct 8.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\Nearshore Rotifers\Ontario\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E680D374-9346-4D3C-A966-96718C582167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF98742-DEE0-4DFF-88E3-685464F8C86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EE00D479-7808-1347-B6F9-7D68A252F316}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="3" xr2:uid="{EE00D479-7808-1347-B6F9-7D68A252F316}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot vol biomass" sheetId="5" r:id="rId1"/>
@@ -20,11 +20,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NS cnt'!$A$1:$I$419</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NS sample'!$A$1:$R$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NS sample'!$A$16:$O$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="5" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -451,8 +451,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -473,12 +474,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -486,6 +489,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -534,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -564,6 +568,14 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5317,7 +5329,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BBCF9175-BF6D-CF48-A553-9B221349CD16}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BBCF9175-BF6D-CF48-A553-9B221349CD16}" name="PivotTable3" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:P67" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -5679,7 +5691,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF9B703-39F0-9846-93CF-331A802AE429}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF9B703-39F0-9846-93CF-331A802AE429}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:P67" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -11425,13 +11437,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37AFF009-BBB3-F442-8093-7922CF5C42A3}">
-  <dimension ref="A1:I419"/>
+  <dimension ref="A1:S610"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" customWidth="1"/>
+    <col min="16" max="16" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>97</v>
       </c>
@@ -11459,8 +11474,12 @@
       <c r="I1" s="17" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -11489,7 +11508,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -11518,7 +11537,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -11547,7 +11566,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -11576,7 +11595,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -11605,7 +11624,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -11634,7 +11653,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -11663,7 +11682,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -11692,7 +11711,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -11721,7 +11740,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -11750,7 +11769,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -11779,7 +11798,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -11808,7 +11827,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -11837,7 +11856,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -11866,7 +11885,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -16999,7 +17018,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>31</v>
       </c>
@@ -17027,8 +17046,11 @@
       <c r="I193" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q193">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>31</v>
       </c>
@@ -17056,8 +17078,11 @@
       <c r="I194" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q194">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>31</v>
       </c>
@@ -17085,8 +17110,11 @@
       <c r="I195" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q195">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>31</v>
       </c>
@@ -17114,8 +17142,11 @@
       <c r="I196" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q196">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>31</v>
       </c>
@@ -17143,8 +17174,11 @@
       <c r="I197" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q197">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>35</v>
       </c>
@@ -17172,8 +17206,11 @@
       <c r="I198" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q198">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>35</v>
       </c>
@@ -17201,8 +17238,11 @@
       <c r="I199" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q199">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>35</v>
       </c>
@@ -17230,8 +17270,11 @@
       <c r="I200" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q200">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>35</v>
       </c>
@@ -17259,8 +17302,11 @@
       <c r="I201" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q201">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>35</v>
       </c>
@@ -17288,8 +17334,11 @@
       <c r="I202" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q202">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>35</v>
       </c>
@@ -17317,8 +17366,11 @@
       <c r="I203" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q203">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>35</v>
       </c>
@@ -17346,8 +17398,11 @@
       <c r="I204" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q204">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>35</v>
       </c>
@@ -17375,8 +17430,11 @@
       <c r="I205" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q205">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>35</v>
       </c>
@@ -17404,8 +17462,11 @@
       <c r="I206" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q206">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>35</v>
       </c>
@@ -17433,8 +17494,11 @@
       <c r="I207" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q207">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>35</v>
       </c>
@@ -17462,8 +17526,11 @@
       <c r="I208" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q208">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>35</v>
       </c>
@@ -17491,8 +17558,11 @@
       <c r="I209" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q209">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>35</v>
       </c>
@@ -17520,8 +17590,11 @@
       <c r="I210" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q210">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="211" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>35</v>
       </c>
@@ -17549,8 +17622,11 @@
       <c r="I211" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q211">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="212" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>35</v>
       </c>
@@ -17578,8 +17654,11 @@
       <c r="I212" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q212">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>35</v>
       </c>
@@ -17607,8 +17686,11 @@
       <c r="I213" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q213">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>35</v>
       </c>
@@ -17636,8 +17718,11 @@
       <c r="I214" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q214">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="215" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>35</v>
       </c>
@@ -17665,8 +17750,11 @@
       <c r="I215" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q215">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="216" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>35</v>
       </c>
@@ -17694,8 +17782,11 @@
       <c r="I216" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q216">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="217" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>35</v>
       </c>
@@ -17723,8 +17814,11 @@
       <c r="I217" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q217">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="218" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>35</v>
       </c>
@@ -17752,8 +17846,11 @@
       <c r="I218" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q218">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>35</v>
       </c>
@@ -17781,8 +17878,11 @@
       <c r="I219" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q219">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>35</v>
       </c>
@@ -17810,8 +17910,11 @@
       <c r="I220" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q220">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>35</v>
       </c>
@@ -17839,8 +17942,11 @@
       <c r="I221" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q221">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>35</v>
       </c>
@@ -17868,8 +17974,11 @@
       <c r="I222" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q222">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="223" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>35</v>
       </c>
@@ -17897,8 +18006,11 @@
       <c r="I223" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q223">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>35</v>
       </c>
@@ -17926,8 +18038,11 @@
       <c r="I224" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q224">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>35</v>
       </c>
@@ -17955,8 +18070,11 @@
       <c r="I225" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q225">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="226" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>35</v>
       </c>
@@ -17984,8 +18102,11 @@
       <c r="I226" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q226">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>36</v>
       </c>
@@ -18013,8 +18134,11 @@
       <c r="I227" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q227">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>36</v>
       </c>
@@ -18042,8 +18166,11 @@
       <c r="I228" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q228">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>36</v>
       </c>
@@ -18071,8 +18198,11 @@
       <c r="I229" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q229">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="230" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>36</v>
       </c>
@@ -18100,8 +18230,11 @@
       <c r="I230" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q230">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="231" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>36</v>
       </c>
@@ -18129,8 +18262,11 @@
       <c r="I231" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q231">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="232" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>36</v>
       </c>
@@ -18158,8 +18294,11 @@
       <c r="I232" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q232">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="233" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>36</v>
       </c>
@@ -18187,8 +18326,11 @@
       <c r="I233" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q233">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="234" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>36</v>
       </c>
@@ -18216,8 +18358,11 @@
       <c r="I234" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q234">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="235" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>36</v>
       </c>
@@ -18245,8 +18390,11 @@
       <c r="I235" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q235">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="236" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>36</v>
       </c>
@@ -18274,8 +18422,11 @@
       <c r="I236" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q236">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="237" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>36</v>
       </c>
@@ -18303,8 +18454,11 @@
       <c r="I237" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q237">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="238" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>36</v>
       </c>
@@ -18332,8 +18486,11 @@
       <c r="I238" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q238">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="239" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>36</v>
       </c>
@@ -18361,8 +18518,11 @@
       <c r="I239" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q239">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="240" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>36</v>
       </c>
@@ -18390,8 +18550,11 @@
       <c r="I240" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q240">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="241" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>36</v>
       </c>
@@ -18419,8 +18582,11 @@
       <c r="I241" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q241">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="242" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>36</v>
       </c>
@@ -18448,8 +18614,11 @@
       <c r="I242" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q242">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="243" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>36</v>
       </c>
@@ -18477,8 +18646,11 @@
       <c r="I243" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q243">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="244" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>36</v>
       </c>
@@ -18506,8 +18678,11 @@
       <c r="I244" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q244">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="245" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>36</v>
       </c>
@@ -18535,8 +18710,11 @@
       <c r="I245" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q245">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="246" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>36</v>
       </c>
@@ -18564,8 +18742,11 @@
       <c r="I246" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q246">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="247" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>36</v>
       </c>
@@ -18593,8 +18774,11 @@
       <c r="I247" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q247">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="248" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>36</v>
       </c>
@@ -18622,8 +18806,11 @@
       <c r="I248" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q248">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="249" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>36</v>
       </c>
@@ -18651,8 +18838,11 @@
       <c r="I249" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q249">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="250" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>36</v>
       </c>
@@ -18680,8 +18870,11 @@
       <c r="I250" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q250">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="251" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>36</v>
       </c>
@@ -18709,8 +18902,11 @@
       <c r="I251" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q251">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="252" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>36</v>
       </c>
@@ -18738,8 +18934,11 @@
       <c r="I252" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q252">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="253" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>36</v>
       </c>
@@ -18767,8 +18966,11 @@
       <c r="I253" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q253">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="254" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>36</v>
       </c>
@@ -18796,8 +18998,11 @@
       <c r="I254" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q254">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="255" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>36</v>
       </c>
@@ -18825,8 +19030,11 @@
       <c r="I255" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q255">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="256" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>36</v>
       </c>
@@ -18854,8 +19062,11 @@
       <c r="I256" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q256">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="257" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>36</v>
       </c>
@@ -18883,8 +19094,11 @@
       <c r="I257" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q257">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="258" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>36</v>
       </c>
@@ -18912,8 +19126,11 @@
       <c r="I258" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q258">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="259" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>36</v>
       </c>
@@ -18941,8 +19158,11 @@
       <c r="I259" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q259">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="260" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>37</v>
       </c>
@@ -18970,8 +19190,11 @@
       <c r="I260" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q260">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="261" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>37</v>
       </c>
@@ -18999,8 +19222,11 @@
       <c r="I261" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q261">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="262" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>37</v>
       </c>
@@ -19028,8 +19254,11 @@
       <c r="I262" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q262">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="263" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>37</v>
       </c>
@@ -19057,8 +19286,11 @@
       <c r="I263" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q263">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="264" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>37</v>
       </c>
@@ -19086,8 +19318,11 @@
       <c r="I264" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q264">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="265" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>37</v>
       </c>
@@ -19115,8 +19350,11 @@
       <c r="I265" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q265">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="266" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>37</v>
       </c>
@@ -19144,8 +19382,11 @@
       <c r="I266" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q266">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="267" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>37</v>
       </c>
@@ -19173,8 +19414,11 @@
       <c r="I267" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q267">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="268" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>37</v>
       </c>
@@ -19202,8 +19446,11 @@
       <c r="I268" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q268">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="269" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>37</v>
       </c>
@@ -19231,8 +19478,11 @@
       <c r="I269" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q269">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="270" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>37</v>
       </c>
@@ -19260,8 +19510,11 @@
       <c r="I270" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q270">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="271" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>37</v>
       </c>
@@ -19289,8 +19542,11 @@
       <c r="I271" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q271">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="272" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>37</v>
       </c>
@@ -19318,8 +19574,11 @@
       <c r="I272" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q272">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="273" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>37</v>
       </c>
@@ -19347,8 +19606,11 @@
       <c r="I273" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q273">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="274" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>37</v>
       </c>
@@ -19376,8 +19638,11 @@
       <c r="I274" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q274">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="275" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>37</v>
       </c>
@@ -19405,8 +19670,11 @@
       <c r="I275" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q275">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="276" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>37</v>
       </c>
@@ -19434,8 +19702,11 @@
       <c r="I276" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q276">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="277" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>37</v>
       </c>
@@ -19463,8 +19734,11 @@
       <c r="I277" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q277">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="278" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>37</v>
       </c>
@@ -19492,8 +19766,11 @@
       <c r="I278" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q278">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="279" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>37</v>
       </c>
@@ -19521,8 +19798,11 @@
       <c r="I279" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q279">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="280" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>37</v>
       </c>
@@ -19550,8 +19830,11 @@
       <c r="I280" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q280">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="281" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>37</v>
       </c>
@@ -19579,8 +19862,11 @@
       <c r="I281" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q281">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="282" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>37</v>
       </c>
@@ -19608,8 +19894,11 @@
       <c r="I282" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q282">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="283" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>37</v>
       </c>
@@ -19637,8 +19926,11 @@
       <c r="I283" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q283">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="284" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>37</v>
       </c>
@@ -19666,8 +19958,11 @@
       <c r="I284" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q284">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="285" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>37</v>
       </c>
@@ -19695,8 +19990,11 @@
       <c r="I285" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q285">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="286" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>37</v>
       </c>
@@ -19724,8 +20022,11 @@
       <c r="I286" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q286">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="287" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>37</v>
       </c>
@@ -19753,8 +20054,11 @@
       <c r="I287" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q287">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="288" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>37</v>
       </c>
@@ -19782,8 +20086,11 @@
       <c r="I288" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q288">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="289" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>37</v>
       </c>
@@ -19811,8 +20118,11 @@
       <c r="I289" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q289">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="290" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>37</v>
       </c>
@@ -19840,8 +20150,11 @@
       <c r="I290" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q290">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="291" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>37</v>
       </c>
@@ -19869,8 +20182,11 @@
       <c r="I291" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q291">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="292" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>38</v>
       </c>
@@ -19898,8 +20214,11 @@
       <c r="I292" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q292">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="293" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>38</v>
       </c>
@@ -19927,8 +20246,11 @@
       <c r="I293" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q293">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="294" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>38</v>
       </c>
@@ -19956,8 +20278,11 @@
       <c r="I294" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q294">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="295" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>38</v>
       </c>
@@ -19985,8 +20310,11 @@
       <c r="I295" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="296" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q295">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="296" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>38</v>
       </c>
@@ -20014,8 +20342,11 @@
       <c r="I296" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="297" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q296">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="297" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>38</v>
       </c>
@@ -20043,8 +20374,11 @@
       <c r="I297" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="298" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q297">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="298" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>38</v>
       </c>
@@ -20072,8 +20406,11 @@
       <c r="I298" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="299" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q298">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="299" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>38</v>
       </c>
@@ -20101,8 +20438,11 @@
       <c r="I299" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="300" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q299">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="300" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>38</v>
       </c>
@@ -20130,8 +20470,11 @@
       <c r="I300" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="301" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q300">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="301" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>38</v>
       </c>
@@ -20159,8 +20502,11 @@
       <c r="I301" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="302" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q301">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="302" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>38</v>
       </c>
@@ -20188,8 +20534,11 @@
       <c r="I302" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="303" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q302">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="303" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>38</v>
       </c>
@@ -20217,8 +20566,11 @@
       <c r="I303" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="304" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q303">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="304" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>38</v>
       </c>
@@ -20246,8 +20598,11 @@
       <c r="I304" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="305" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q304">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="305" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>38</v>
       </c>
@@ -20275,8 +20630,11 @@
       <c r="I305" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="306" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q305">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="306" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>38</v>
       </c>
@@ -20304,8 +20662,11 @@
       <c r="I306" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="307" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q306">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="307" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>38</v>
       </c>
@@ -20333,8 +20694,11 @@
       <c r="I307" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q307">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="308" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>38</v>
       </c>
@@ -20362,8 +20726,11 @@
       <c r="I308" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q308">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="309" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>38</v>
       </c>
@@ -20391,8 +20758,11 @@
       <c r="I309" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q309">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="310" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>38</v>
       </c>
@@ -20420,8 +20790,11 @@
       <c r="I310" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="311" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q310">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="311" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>38</v>
       </c>
@@ -20449,8 +20822,11 @@
       <c r="I311" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="312" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q311">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="312" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>38</v>
       </c>
@@ -20478,8 +20854,11 @@
       <c r="I312" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="313" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q312">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>38</v>
       </c>
@@ -20507,8 +20886,11 @@
       <c r="I313" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="314" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q313">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>38</v>
       </c>
@@ -20536,8 +20918,11 @@
       <c r="I314" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="315" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q314">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>38</v>
       </c>
@@ -20565,8 +20950,11 @@
       <c r="I315" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="316" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q315">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="316" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>38</v>
       </c>
@@ -20594,8 +20982,11 @@
       <c r="I316" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="317" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q316">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>38</v>
       </c>
@@ -20623,8 +21014,11 @@
       <c r="I317" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="318" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q317">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>38</v>
       </c>
@@ -20652,8 +21046,11 @@
       <c r="I318" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="319" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q318">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="319" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>38</v>
       </c>
@@ -20681,8 +21078,11 @@
       <c r="I319" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="320" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q319">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="320" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>38</v>
       </c>
@@ -20710,8 +21110,11 @@
       <c r="I320" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="321" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q320">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="321" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>38</v>
       </c>
@@ -20739,8 +21142,11 @@
       <c r="I321" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="322" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q321">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="322" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>38</v>
       </c>
@@ -20768,8 +21174,11 @@
       <c r="I322" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q322">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="323" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>39</v>
       </c>
@@ -20797,8 +21206,11 @@
       <c r="I323" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="324" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q323">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="324" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>39</v>
       </c>
@@ -20826,8 +21238,11 @@
       <c r="I324" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="325" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q324">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="325" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>39</v>
       </c>
@@ -20855,8 +21270,11 @@
       <c r="I325" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="326" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q325">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="326" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>39</v>
       </c>
@@ -20884,8 +21302,11 @@
       <c r="I326" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q326">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="327" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>39</v>
       </c>
@@ -20913,8 +21334,11 @@
       <c r="I327" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="328" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q327">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="328" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>39</v>
       </c>
@@ -20942,8 +21366,11 @@
       <c r="I328" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="329" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q328">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="329" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>39</v>
       </c>
@@ -20971,8 +21398,11 @@
       <c r="I329" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="330" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q329">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="330" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>39</v>
       </c>
@@ -21000,8 +21430,11 @@
       <c r="I330" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="331" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q330">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="331" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>39</v>
       </c>
@@ -21029,8 +21462,11 @@
       <c r="I331" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="332" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q331">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="332" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>39</v>
       </c>
@@ -21058,8 +21494,11 @@
       <c r="I332" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="333" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q332">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="333" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>39</v>
       </c>
@@ -21087,8 +21526,11 @@
       <c r="I333" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="334" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q333">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="334" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>39</v>
       </c>
@@ -21116,8 +21558,11 @@
       <c r="I334" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="335" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q334">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="335" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>39</v>
       </c>
@@ -21145,8 +21590,11 @@
       <c r="I335" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="336" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q335">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="336" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>39</v>
       </c>
@@ -21174,8 +21622,11 @@
       <c r="I336" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="337" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q336">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="337" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>39</v>
       </c>
@@ -21203,8 +21654,11 @@
       <c r="I337" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="338" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q337">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="338" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>39</v>
       </c>
@@ -21232,8 +21686,11 @@
       <c r="I338" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="339" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q338">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="339" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>39</v>
       </c>
@@ -21261,8 +21718,11 @@
       <c r="I339" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="340" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q339">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="340" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>39</v>
       </c>
@@ -21290,8 +21750,11 @@
       <c r="I340" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="341" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q340">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="341" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>39</v>
       </c>
@@ -21319,8 +21782,11 @@
       <c r="I341" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="342" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q341">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="342" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>39</v>
       </c>
@@ -21348,8 +21814,11 @@
       <c r="I342" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="343" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q342">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="343" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>39</v>
       </c>
@@ -21377,8 +21846,11 @@
       <c r="I343" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="344" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q343">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="344" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>39</v>
       </c>
@@ -21406,8 +21878,11 @@
       <c r="I344" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="345" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q344">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="345" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>39</v>
       </c>
@@ -21435,8 +21910,11 @@
       <c r="I345" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="346" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q345">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="346" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>39</v>
       </c>
@@ -21464,8 +21942,11 @@
       <c r="I346" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="347" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q346">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="347" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>39</v>
       </c>
@@ -21493,8 +21974,11 @@
       <c r="I347" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="348" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q347">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="348" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>39</v>
       </c>
@@ -21522,8 +22006,11 @@
       <c r="I348" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="349" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q348">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="349" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>39</v>
       </c>
@@ -21551,8 +22038,11 @@
       <c r="I349" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="350" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q349">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="350" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>39</v>
       </c>
@@ -21580,8 +22070,11 @@
       <c r="I350" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="351" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q350">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="351" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>39</v>
       </c>
@@ -21609,8 +22102,11 @@
       <c r="I351" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="352" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q351">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="352" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>39</v>
       </c>
@@ -21638,8 +22134,11 @@
       <c r="I352" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="353" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q352">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="353" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>39</v>
       </c>
@@ -21667,8 +22166,11 @@
       <c r="I353" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="354" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q353">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="354" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>40</v>
       </c>
@@ -21696,8 +22198,11 @@
       <c r="I354" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="355" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q354">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="355" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>40</v>
       </c>
@@ -21725,8 +22230,11 @@
       <c r="I355" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="356" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q355">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="356" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>40</v>
       </c>
@@ -21754,8 +22262,11 @@
       <c r="I356" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="357" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q356">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="357" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>40</v>
       </c>
@@ -21783,8 +22294,11 @@
       <c r="I357" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="358" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q357">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="358" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>40</v>
       </c>
@@ -21812,8 +22326,11 @@
       <c r="I358" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="359" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q358">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="359" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>40</v>
       </c>
@@ -21841,8 +22358,11 @@
       <c r="I359" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="360" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q359">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="360" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>40</v>
       </c>
@@ -21870,8 +22390,11 @@
       <c r="I360" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="361" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q360">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="361" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>40</v>
       </c>
@@ -21899,8 +22422,11 @@
       <c r="I361" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="362" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q361">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="362" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>40</v>
       </c>
@@ -21928,8 +22454,11 @@
       <c r="I362" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="363" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q362">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="363" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>40</v>
       </c>
@@ -21957,8 +22486,11 @@
       <c r="I363" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="364" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q363">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="364" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>40</v>
       </c>
@@ -21986,8 +22518,11 @@
       <c r="I364" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="365" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q364">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="365" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>40</v>
       </c>
@@ -22015,8 +22550,11 @@
       <c r="I365" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="366" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q365">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="366" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>40</v>
       </c>
@@ -22044,8 +22582,11 @@
       <c r="I366" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="367" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q366">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="367" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>40</v>
       </c>
@@ -22073,8 +22614,11 @@
       <c r="I367" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="368" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q367">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="368" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>40</v>
       </c>
@@ -22102,8 +22646,11 @@
       <c r="I368" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="369" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q368">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="369" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>40</v>
       </c>
@@ -22131,8 +22678,11 @@
       <c r="I369" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="370" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q369">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="370" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>40</v>
       </c>
@@ -22160,8 +22710,11 @@
       <c r="I370" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="371" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q370">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="371" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>40</v>
       </c>
@@ -22189,8 +22742,11 @@
       <c r="I371" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="372" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q371">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="372" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>40</v>
       </c>
@@ -22218,8 +22774,11 @@
       <c r="I372" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="373" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q372">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="373" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>40</v>
       </c>
@@ -22247,8 +22806,11 @@
       <c r="I373" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="374" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q373">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="374" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>40</v>
       </c>
@@ -22276,8 +22838,11 @@
       <c r="I374" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="375" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q374">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="375" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>40</v>
       </c>
@@ -22305,8 +22870,11 @@
       <c r="I375" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="376" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q375">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="376" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>40</v>
       </c>
@@ -22334,8 +22902,11 @@
       <c r="I376" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="377" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q376">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="377" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>40</v>
       </c>
@@ -22363,8 +22934,11 @@
       <c r="I377" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="378" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q377">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="378" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>40</v>
       </c>
@@ -22392,8 +22966,11 @@
       <c r="I378" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="379" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q378">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="379" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>40</v>
       </c>
@@ -22421,8 +22998,11 @@
       <c r="I379" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="380" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q379">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="380" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>40</v>
       </c>
@@ -22450,8 +23030,11 @@
       <c r="I380" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="381" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q380">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="381" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>40</v>
       </c>
@@ -22479,8 +23062,11 @@
       <c r="I381" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="382" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q381">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="382" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>40</v>
       </c>
@@ -22508,8 +23094,11 @@
       <c r="I382" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="383" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q382">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="383" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>40</v>
       </c>
@@ -22537,8 +23126,11 @@
       <c r="I383" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="384" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q383">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="384" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
         <v>40</v>
       </c>
@@ -22566,8 +23158,11 @@
       <c r="I384" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="385" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q384">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="385" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>41</v>
       </c>
@@ -22595,8 +23190,11 @@
       <c r="I385" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="386" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q385">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="386" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
         <v>41</v>
       </c>
@@ -22624,8 +23222,11 @@
       <c r="I386" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="387" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q386">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="387" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
         <v>41</v>
       </c>
@@ -22653,8 +23254,11 @@
       <c r="I387" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="388" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q387">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="388" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
         <v>41</v>
       </c>
@@ -22682,8 +23286,11 @@
       <c r="I388" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="389" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q388">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="389" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
         <v>41</v>
       </c>
@@ -22711,8 +23318,11 @@
       <c r="I389" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="390" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q389">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="390" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
         <v>41</v>
       </c>
@@ -22740,8 +23350,11 @@
       <c r="I390" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="391" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q390">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="391" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
         <v>41</v>
       </c>
@@ -22769,8 +23382,11 @@
       <c r="I391" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="392" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q391">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="392" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
         <v>41</v>
       </c>
@@ -22798,8 +23414,11 @@
       <c r="I392" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="393" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q392">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="393" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
         <v>41</v>
       </c>
@@ -22827,8 +23446,11 @@
       <c r="I393" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="394" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q393">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="394" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
         <v>41</v>
       </c>
@@ -22856,8 +23478,11 @@
       <c r="I394" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="395" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q394">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="395" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
         <v>41</v>
       </c>
@@ -22885,8 +23510,11 @@
       <c r="I395" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="396" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q395">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="396" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
         <v>41</v>
       </c>
@@ -22914,8 +23542,11 @@
       <c r="I396" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="397" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q396">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="397" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
         <v>41</v>
       </c>
@@ -22943,8 +23574,11 @@
       <c r="I397" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="398" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q397">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="398" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
         <v>41</v>
       </c>
@@ -22972,8 +23606,11 @@
       <c r="I398" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="399" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q398">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="399" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
         <v>41</v>
       </c>
@@ -23001,8 +23638,11 @@
       <c r="I399" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="400" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q399">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="400" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
         <v>41</v>
       </c>
@@ -23030,8 +23670,11 @@
       <c r="I400" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="401" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q400">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="401" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>41</v>
       </c>
@@ -23059,8 +23702,11 @@
       <c r="I401" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="402" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q401">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="402" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>41</v>
       </c>
@@ -23088,8 +23734,11 @@
       <c r="I402" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="403" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q402">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="403" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>41</v>
       </c>
@@ -23117,8 +23766,11 @@
       <c r="I403" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="404" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q403">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="404" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>41</v>
       </c>
@@ -23146,8 +23798,11 @@
       <c r="I404" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="405" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q404">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="405" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>41</v>
       </c>
@@ -23175,8 +23830,11 @@
       <c r="I405" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="406" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q405">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="406" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>41</v>
       </c>
@@ -23204,8 +23862,11 @@
       <c r="I406" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="407" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q406">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="407" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>41</v>
       </c>
@@ -23233,8 +23894,11 @@
       <c r="I407" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="408" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q407">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="408" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>41</v>
       </c>
@@ -23262,8 +23926,11 @@
       <c r="I408" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="409" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q408">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="409" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>41</v>
       </c>
@@ -23291,8 +23958,11 @@
       <c r="I409" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="410" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q409">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="410" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
         <v>41</v>
       </c>
@@ -23320,8 +23990,11 @@
       <c r="I410" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="411" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q410">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="411" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
         <v>41</v>
       </c>
@@ -23349,8 +24022,11 @@
       <c r="I411" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="412" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q411">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="412" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
         <v>41</v>
       </c>
@@ -23378,8 +24054,11 @@
       <c r="I412" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="413" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q412">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="413" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
         <v>41</v>
       </c>
@@ -23407,8 +24086,11 @@
       <c r="I413" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="414" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q413">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="414" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
         <v>41</v>
       </c>
@@ -23436,8 +24118,11 @@
       <c r="I414" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="415" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q414">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="415" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
         <v>41</v>
       </c>
@@ -23465,8 +24150,11 @@
       <c r="I415" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="416" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q415">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="416" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
         <v>41</v>
       </c>
@@ -23494,8 +24182,11 @@
       <c r="I416" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="417" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q416">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="417" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
         <v>41</v>
       </c>
@@ -23523,8 +24214,11 @@
       <c r="I417" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="418" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q417">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="418" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
         <v>41</v>
       </c>
@@ -23552,8 +24246,11 @@
       <c r="I418" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="419" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="Q418">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="419" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
         <v>41</v>
       </c>
@@ -23581,19 +24278,976 @@
       <c r="I419" t="s">
         <v>45</v>
       </c>
+      <c r="Q419">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="420" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q420">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="421" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q421">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="422" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q422">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="423" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q423">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="424" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q424">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="425" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q425">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="426" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q426">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="427" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q427">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="428" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q428">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="429" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q429">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="430" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q430">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="431" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q431">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="432" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q432">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="433" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q433">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="434" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q434">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="435" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q435">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="436" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q436">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="437" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q437">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="438" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q438">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="439" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q439">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="440" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q440">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="441" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q441">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="442" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q442">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="443" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q443">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="444" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q444">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="445" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q445">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="446" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q446">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="447" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q447">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="448" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q448">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="449" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q449">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="450" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q450">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="451" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q451">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="452" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q452">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="453" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q453">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="454" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q454">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="455" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q455">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="456" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q456">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="457" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q457">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="458" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q458">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="459" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q459">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="460" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q460">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="461" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q461">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="462" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q462">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="463" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q463">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="464" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q464">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="465" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q465">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="466" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q466">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="467" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q467">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="468" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q468">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="469" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q469">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="470" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q470">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="471" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q471">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="472" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q472">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="473" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q473">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="474" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q474">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="475" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q475">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="476" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q476">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="477" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q477">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="478" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q478">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="479" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q479">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="480" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q480">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="481" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q481">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="482" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q482">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="483" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q483">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="484" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q484">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="485" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q485">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="486" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q486">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="487" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q487">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="488" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q488">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="489" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q489">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="490" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q490">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="491" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q491">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="492" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q492">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="493" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q493">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="494" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q494">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="495" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q495">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="496" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q496">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="497" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q497">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="498" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q498">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="499" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q499">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="500" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q500">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="501" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q501">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="502" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q502">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="503" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q503">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="504" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q504">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="505" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q505">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="506" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q506">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="507" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q507">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="508" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q508">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="509" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q509">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="510" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q510">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="511" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q511">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="512" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q512">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="513" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q513">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="514" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q514">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="515" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q515">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="516" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q516">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="517" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q517">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="518" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q518">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="519" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q519">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="520" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q520">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="521" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q521">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="522" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q522">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="523" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q523">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="524" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q524">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="525" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q525">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="526" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q526">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="527" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q527">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="528" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q528">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="529" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q529">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="530" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q530">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="531" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q531">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="532" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q532">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="533" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q533">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="534" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q534">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="535" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q535">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="536" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q536">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="537" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q537">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="538" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q538">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="539" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q539">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="540" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q540">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="541" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q541">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="542" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q542">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="543" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q543">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="544" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q544">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="545" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q545">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="546" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q546">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="547" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q547">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="548" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q548">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="549" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q549">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="550" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q550">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="551" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q551">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="552" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q552">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="553" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q553">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="554" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q554">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="555" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q555">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="556" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q556">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="557" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q557">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="558" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q558">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="559" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q559">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="560" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q560">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="561" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q561">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="562" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q562">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="563" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q563">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="564" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q564">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="565" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q565">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="566" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q566">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="567" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q567">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="568" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q568">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="569" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q569">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="570" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q570">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="571" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q571">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="572" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q572">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="573" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q573">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="574" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q574">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="575" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q575">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="576" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q576">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="577" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q577">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="578" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q578">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="579" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q579">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="580" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q580">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="581" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q581">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="582" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q582">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="583" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q583">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="584" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q584">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="585" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q585">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="586" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q586">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="587" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q587">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="588" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q588">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="589" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q589">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="590" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q590">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="591" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q591">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="592" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q592">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="593" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q593">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="594" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q594">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="595" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q595">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="596" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q596">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="597" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q597">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="598" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q598">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="599" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q599">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="600" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q600">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="601" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q601">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="602" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q602">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="603" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q603">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="604" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q604">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="605" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q605">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="606" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q606">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="607" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q607">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="608" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q608">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="609" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q609">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="610" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q610">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I419" xr:uid="{37AFF009-BBB3-F442-8093-7922CF5C42A3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFCE812-0050-204D-B1ED-4803A232C5AA}">
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:AC50"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>97</v>
       </c>
@@ -23649,7 +25303,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -23708,7 +25362,7 @@
         <v>-76.951549999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -23767,7 +25421,7 @@
         <v>-79.417216666666661</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -23826,7 +25480,7 @@
         <v>-78.999750000000006</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>29</v>
       </c>
@@ -23885,7 +25539,7 @@
         <v>-78.730166666666662</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>30</v>
       </c>
@@ -23944,7 +25598,7 @@
         <v>-77.989850000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
@@ -24003,7 +25657,7 @@
         <v>-77.1584</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>35</v>
       </c>
@@ -24062,7 +25716,7 @@
         <v>-76.734133333333332</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
@@ -24121,7 +25775,7 @@
         <v>-76.789333333333332</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
@@ -24180,7 +25834,7 @@
         <v>-76.287033333333326</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>38</v>
       </c>
@@ -24239,7 +25893,7 @@
         <v>-78.868566666666666</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>39</v>
       </c>
@@ -24298,7 +25952,7 @@
         <v>-76.997200000000007</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>40</v>
       </c>
@@ -24357,7 +26011,7 @@
         <v>-78.050116666666668</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>41</v>
       </c>
@@ -24415,6 +26069,254 @@
       <c r="R14" s="12">
         <v>-79.271766666666664</v>
       </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="19"/>
+      <c r="X16" s="19"/>
+      <c r="Y16" s="19"/>
+      <c r="Z16" s="19"/>
+      <c r="AA16" s="19"/>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="21"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="11"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="21"/>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="21"/>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="20"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="19"/>
+      <c r="W28" s="19"/>
+      <c r="X28" s="19"/>
+      <c r="Y28" s="19"/>
+      <c r="Z28" s="19"/>
+      <c r="AA28" s="19"/>
+      <c r="AB28" s="19"/>
+      <c r="AC28" s="19"/>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="L29" s="21"/>
+      <c r="M29" s="22"/>
+      <c r="P29" s="21"/>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="L30" s="21"/>
+      <c r="M30" s="22"/>
+      <c r="P30" s="21"/>
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="L31" s="21"/>
+      <c r="M31" s="22"/>
+      <c r="P31" s="21"/>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="L32" s="21"/>
+      <c r="M32" s="22"/>
+      <c r="P32" s="21"/>
+    </row>
+    <row r="33" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L33" s="21"/>
+      <c r="M33" s="22"/>
+      <c r="P33" s="21"/>
+    </row>
+    <row r="34" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L34" s="21"/>
+      <c r="M34" s="22"/>
+      <c r="P34" s="21"/>
+    </row>
+    <row r="35" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L35" s="21"/>
+      <c r="M35" s="22"/>
+      <c r="P35" s="21"/>
+    </row>
+    <row r="36" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L36" s="21"/>
+      <c r="M36" s="22"/>
+      <c r="P36" s="21"/>
+    </row>
+    <row r="37" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L37" s="21"/>
+      <c r="M37" s="22"/>
+      <c r="P37" s="21"/>
+    </row>
+    <row r="38" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L38" s="21"/>
+      <c r="M38" s="22"/>
+      <c r="P38" s="21"/>
+    </row>
+    <row r="39" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L39" s="21"/>
+      <c r="M39" s="22"/>
+      <c r="P39" s="21"/>
+    </row>
+    <row r="40" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L40" s="21"/>
+      <c r="M40" s="22"/>
+      <c r="P40" s="21"/>
+    </row>
+    <row r="41" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L41" s="21"/>
+      <c r="M41" s="22"/>
+      <c r="P41" s="21"/>
+    </row>
+    <row r="42" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L42" s="21"/>
+      <c r="M42" s="22"/>
+      <c r="P42" s="21"/>
+    </row>
+    <row r="43" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L43" s="21"/>
+      <c r="M43" s="22"/>
+      <c r="P43" s="21"/>
+    </row>
+    <row r="44" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L44" s="21"/>
+      <c r="M44" s="22"/>
+      <c r="P44" s="21"/>
+    </row>
+    <row r="45" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L45" s="21"/>
+      <c r="M45" s="22"/>
+      <c r="P45" s="21"/>
+    </row>
+    <row r="46" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L46" s="21"/>
+      <c r="M46" s="22"/>
+      <c r="P46" s="21"/>
+    </row>
+    <row r="47" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L47" s="21"/>
+      <c r="M47" s="22"/>
+      <c r="P47" s="21"/>
+    </row>
+    <row r="48" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L48" s="21"/>
+      <c r="M48" s="22"/>
+      <c r="P48" s="21"/>
+    </row>
+    <row r="49" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L49" s="21"/>
+      <c r="M49" s="22"/>
+      <c r="P49" s="21"/>
+    </row>
+    <row r="50" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L50" s="21"/>
+      <c r="M50" s="22"/>
+      <c r="P50" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>